<commit_message>
new demand and emissions figure
</commit_message>
<xml_diff>
--- a/Results/Chemical industry emissions.xlsx
+++ b/Results/Chemical industry emissions.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20404"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20405"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\anabera\Desktop\Ongoing projects\Prospective LCA\Results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73A63116-758E-4A56-B7E9-B3B3EF4F2CA5}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16C14E30-2B3F-4D89-9321-1FE7BE06F2AC}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="14025" activeTab="2" xr2:uid="{B97F3159-796F-4D28-AF5A-4DA070CE1984}"/>
   </bookViews>
@@ -890,16 +890,18 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="B3" s="14">
-        <v>182</v>
-      </c>
-      <c r="C3" s="14">
-        <v>457</v>
+        <v>18</v>
+      </c>
+      <c r="B3" s="15">
+        <f>B2*5</f>
+        <v>500</v>
+      </c>
+      <c r="C3" s="15">
+        <f>C2*5</f>
+        <v>445</v>
       </c>
       <c r="D3" s="14">
-        <v>450</v>
+        <v>355</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -918,18 +920,16 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="19" t="s">
-        <v>18</v>
-      </c>
-      <c r="B5" s="15">
-        <f>B2*5</f>
-        <v>500</v>
-      </c>
-      <c r="C5" s="15">
-        <f>C2*5</f>
-        <v>445</v>
+        <v>17</v>
+      </c>
+      <c r="B5" s="14">
+        <v>182</v>
+      </c>
+      <c r="C5" s="14">
+        <v>457</v>
       </c>
       <c r="D5" s="14">
-        <v>355</v>
+        <v>450</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -937,15 +937,15 @@
         <v>19</v>
       </c>
       <c r="B6" s="15">
-        <f>B5*'Emissions 2050'!E9</f>
+        <f>B3*'Emissions 2050'!E9</f>
         <v>-592.15017899385589</v>
       </c>
       <c r="C6" s="15">
-        <f>C5*'Emissions 2050'!C9</f>
+        <f>C3*'Emissions 2050'!C9</f>
         <v>789.1398488144074</v>
       </c>
       <c r="D6" s="15">
-        <f>D5*'Emissions 2050'!D9</f>
+        <f>D3*'Emissions 2050'!D9</f>
         <v>164.79216746574841</v>
       </c>
     </row>
@@ -954,15 +954,15 @@
         <v>20</v>
       </c>
       <c r="B7" s="15">
-        <f>B5*'Emissions 2050'!E10</f>
+        <f>B3*'Emissions 2050'!E10</f>
         <v>-685.58569963752905</v>
       </c>
       <c r="C7" s="15">
-        <f>C5*'Emissions 2050'!C10</f>
+        <f>C3*'Emissions 2050'!C10</f>
         <v>513.55728461101455</v>
       </c>
       <c r="D7" s="15">
-        <f>D5*'Emissions 2050'!D10</f>
+        <f>D3*'Emissions 2050'!D10</f>
         <v>86.075948957690926</v>
       </c>
     </row>
@@ -971,15 +971,15 @@
         <v>21</v>
       </c>
       <c r="B8" s="15">
-        <f>B5*'Emissions 2050'!E11</f>
+        <f>B3*'Emissions 2050'!E11</f>
         <v>-437.70406457422655</v>
       </c>
       <c r="C8" s="15">
-        <f>C5*'Emissions 2050'!C11</f>
+        <f>C3*'Emissions 2050'!C11</f>
         <v>1218.752561613959</v>
       </c>
       <c r="D8" s="15">
-        <f>D5*'Emissions 2050'!D11</f>
+        <f>D3*'Emissions 2050'!D11</f>
         <v>300.25167049638441</v>
       </c>
     </row>

</xml_diff>